<commit_message>
Reprice to Foundation $997 / Full Presence $1,497; flat $100-$125 setter pay; update scripts, contract, offer and workbook
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N397dYkWM163YQMqrsVR2H
</commit_message>
<xml_diff>
--- a/agency/Vanguard-Outreach-System.xlsx
+++ b/agency/Vanguard-Outreach-System.xlsx
@@ -1203,7 +1203,7 @@
       </c>
       <c r="F5" s="10" t="inlineStr">
         <is>
-          <t>You are my lead scout for Vanguard, a web studio that builds websites for US local businesses (about $2,000 one-time, live within 14 days of kick-off, free demo first).
+          <t>You are my lead scout for Vanguard, a web studio that builds websites for US local businesses (about $1,000 one-time, live within 14 days of kick-off, free demo first).
 1. Using the Outlook (Mailbox) connector, make ONE search_emails call: from "f5bot", since yesterday's date, limit 25. The mailbox is on a free plan of 5 calls per day, so use at most 3 more calls in total (read_email only when a preview has no post link). Never send, move or delete email.
 2. From the alerts, collect every Reddit post or comment URL.
 3. For each URL, fetch the post (try the URL with ".json" on the end, or old.reddit.com). Skip anything older than 72 hours, locked, or already answered by a hired designer.
@@ -1242,7 +1242,7 @@
       </c>
       <c r="F6" s="10" t="inlineStr">
         <is>
-          <t>Open https://www.linkedin.com/messaging/ in a new tab. I run Vanguard, a web studio that builds websites for US local businesses (about $2,000 one-time, live within 14 days of kick-off, free demo first).
+          <t>Open https://www.linkedin.com/messaging/ in a new tab. I run Vanguard, a web studio that builds websites for US local businesses (about $1,000 one-time, live within 14 days of kick-off, free demo first).
 1. Open every conversation that is unread, or where the other person wrote last in the past 7 days.
 2. For each one, classify the reply:
 Reply types (pick one per conversation):
@@ -1251,14 +1251,14 @@
 4. Also check My Network → Invitations (list them, do not accept or decline) and Notifications for comments on my posts that need an answer.
 5. Output a table: name, company, reply type, their last message (one line), my drafted reply, next stage, follow-up date.
 Reply Playbook:
-- Price question → "Fair question. It depends on what you need, but most of our builds land around $2,000, one-time, and the demo is free. Want me to put one together so you can see what you'd get?"
+- Price question → "Fair question. It depends on what you need, but most of our builds land around $1,000, one-time, and the demo is free. Want me to put one together so you can see what you'd get?"
 - Send info → share two portfolio links and offer a free demo for their business.
 - Wants demo → ask for business name + any page; promise the demo within 48 hours, then book a 15-min walkthrough: [Calendly link].
 - Not now → ask when to check back; set the follow-up date.
 - Has a website → offer a free 3-point review, no pressure.
 - Referral → thank them and ask for an intro.
 - Not interested / Opt-out → one polite line, then mark Do-Not-Contact.
-Rules: never send, post, comment, connect, accept or decline anything without my approval in this chat. Never invent facts about a prospect or about Vanguard. Prices: only the ballpark "most of our builds land around $2,000, one-time; the demo is free". Anyone who says stop / not interested / remove me goes on the Do-Not-Contact list and gets no further outreach.</t>
+Rules: never send, post, comment, connect, accept or decline anything without my approval in this chat. Never invent facts about a prospect or about Vanguard. Prices: only the ballpark "most of our builds land around $1,000, one-time; the demo is free". Anyone who says stop / not interested / remove me goes on the Do-Not-Contact list and gets no further outreach.</t>
         </is>
       </c>
     </row>
@@ -1297,7 +1297,7 @@
 Search People with: titles Owner / Founder / Co-owner; company size 1–10; locations from my target list [CITIES]; industries: personal care, wellness and fitness, construction, automotive, restaurants, retail, pet services. Also find up to 5 referral partners in the same cities: bookkeepers, accountants, business coaches, photographers, print/sign shops, marketing freelancers who don't build websites.
 Skip anyone I'm already connected with or have a pending invite to.
 For each person: name, title, business, city, profile link, whether their business has a website (check the company page or a quick Google search), and one personalised first message to send after they accept (under 60 words, mentions one real detail, offers a free demo for owners or a referral swap for partners).
-Output: two tables (A and B), ready for me to action. Rules: never send, post, comment, connect, accept or decline anything without my approval in this chat. Never invent facts about a prospect or about Vanguard. Prices: only the ballpark "most of our builds land around $2,000, one-time; the demo is free". Anyone who says stop / not interested / remove me goes on the Do-Not-Contact list and gets no further outreach.</t>
+Output: two tables (A and B), ready for me to action. Rules: never send, post, comment, connect, accept or decline anything without my approval in this chat. Never invent facts about a prospect or about Vanguard. Prices: only the ballpark "most of our builds land around $1,000, one-time; the demo is free". Anyone who says stop / not interested / remove me goes on the Do-Not-Contact list and gets no further outreach.</t>
         </is>
       </c>
     </row>
@@ -1329,7 +1329,7 @@
       </c>
       <c r="F8" s="10" t="inlineStr">
         <is>
-          <t>Do my Facebook sweep for Vanguard (websites for US local businesses, about $2,000 one-time, free demo first). Do not post, comment, react, add friends or message anyone.
+          <t>Do my Facebook sweep for Vanguard (websites for US local businesses, about $1,000 one-time, free demo first). Do not post, comment, react, add friends or message anyone.
 1. Messenger: open https://www.facebook.com/messages/ including Message Requests. For each unread thread or one where they wrote last, classify the reply:
 Reply types (pick one per conversation):
 Interested · Price question · Send info · Wants demo · Not now · Has a website · Referral · Partner · Not interested · Opt-out · Auto-reply · Wrong person · Booked · Who are you
@@ -1337,7 +1337,7 @@
 2. Groups: open each group in my list [GROUP LINKS]. In each, search for posts from the last 48 hours containing: website, web designer, web developer, recommend, anyone know, need a site. Read the group rules once and note whether service offers are allowed.
 3. For each post where someone needs a website or asks for a recommendation: group, author, link, what they need, a drafted public comment (helpful, says who I am, offers a free demo) and a drafted follow-up DM. Only draft a DM where they asked publicly or invited DMs.
 4. List up to 10 other posts by local business owners where a genuinely helpful comment would fit (questions about getting more customers, Google reviews, booking, marketing), with a drafted comment that gives value and does not pitch.
-Output three tables: Messenger replies, Website requests, Value comments. Rules: never send, post, comment, connect, accept or decline anything without my approval in this chat. Never invent facts about a prospect or about Vanguard. Prices: only the ballpark "most of our builds land around $2,000, one-time; the demo is free". Anyone who says stop / not interested / remove me goes on the Do-Not-Contact list and gets no further outreach.</t>
+Output three tables: Messenger replies, Website requests, Value comments. Rules: never send, post, comment, connect, accept or decline anything without my approval in this chat. Never invent facts about a prospect or about Vanguard. Prices: only the ballpark "most of our builds land around $1,000, one-time; the demo is free". Anyone who says stop / not interested / remove me goes on the Do-Not-Contact list and gets no further outreach.</t>
         </is>
       </c>
     </row>
@@ -1377,7 +1377,7 @@
 3. Opt-outs ("stop", "remove me", "unsubscribe", angry replies): do not draft a reply; list them so I can add them to the suppression list today.
 4. Auto-replies: note the return date as the next follow-up date.
 5. Output a table: sender, business, reply type, one-line summary, drafted reply, next stage, follow-up date. Also report today's numbers if the tool shows them: sent, opens if tracked, replies, bounces.
-Rules: never send, post, comment, connect, accept or decline anything without my approval in this chat. Never invent facts about a prospect or about Vanguard. Prices: only the ballpark "most of our builds land around $2,000, one-time; the demo is free". Anyone who says stop / not interested / remove me goes on the Do-Not-Contact list and gets no further outreach.</t>
+Rules: never send, post, comment, connect, accept or decline anything without my approval in this chat. Never invent facts about a prospect or about Vanguard. Prices: only the ballpark "most of our builds land around $1,000, one-time; the demo is free". Anyone who says stop / not interested / remove me goes on the Do-Not-Contact list and gets no further outreach.</t>
         </is>
       </c>
     </row>
@@ -4264,11 +4264,11 @@
         </is>
       </c>
       <c r="B16" s="26" t="n">
-        <v>2000</v>
+        <v>997</v>
       </c>
       <c r="G16" s="10" t="inlineStr">
         <is>
-          <t>Your stated average project.</t>
+          <t>Foundation price; raise toward $1,497 as more clients take Full Presence.</t>
         </is>
       </c>
     </row>
@@ -17182,7 +17182,7 @@
       </c>
       <c r="C6" s="10" t="inlineStr">
         <is>
-          <t>Honest ballpark: most builds land around $2,000, one-time; the demo is free. Then offer the demo. Never quote exact prices, discounts or payment plans in DMs.</t>
+          <t>Honest ballpark: most builds land around $1,000, one-time; the demo is free. Then offer the demo. Never quote exact prices, discounts or payment plans in DMs.</t>
         </is>
       </c>
       <c r="D6" s="10" t="inlineStr">
@@ -17929,7 +17929,7 @@
       <c r="D17" s="10" t="inlineStr">
         <is>
           <t>Subject: Re: [Business] website idea
-Hi [First name], the question owners ask most is cost. Most of our builds land around $2,000, one-time, live within 14 days of kick-off, and the demo is free either way. Worth 15 minutes? [Calendly link]</t>
+Hi [First name], the question owners ask most is cost. Most of our builds land around $1,000, one-time, live within 14 days of kick-off, and the demo is free either way. Worth 15 minutes? [Calendly link]</t>
         </is>
       </c>
     </row>
@@ -18019,7 +18019,7 @@
       </c>
       <c r="D21" s="10" t="inlineStr">
         <is>
-          <t>Fair question. It depends on what you need, but most of our builds land around $2,000, one-time, and the demo is free. Want me to put one together so you can see what you'd get?</t>
+          <t>Fair question. It depends on what you need, but most of our builds land around $1,000, one-time, and the demo is free. Want me to put one together so you can see what you'd get?</t>
         </is>
       </c>
     </row>

</xml_diff>